<commit_message>
Ground learning examples in five JOP publications and add practical AI resource workflows
</commit_message>
<xml_diff>
--- a/downloads/AI-Use-Log.xlsx
+++ b/downloads/AI-Use-Log.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R8ff0aff7c7334598"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank template" sheetId="2" r:id="Rdd71fe4720134172"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Completed example" sheetId="3" r:id="Rc4bd47aacc804c08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R48303d09f5f94c96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank template" sheetId="2" r:id="Rd1c4011656c642f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Completed example" sheetId="3" r:id="Rb6484603be5c4b8f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -355,7 +355,7 @@
     </x:row>
     <x:row r="2" ht="47" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Dental Research AI • Free, editable Excel worksheet • Version 2 • 8 September 2026</x:v>
+        <x:v>Dental Research AI • Free editable worksheet • Version 3 • 9 September 2026</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -392,7 +392,7 @@
         <x:v>1. Read the example</x:v>
       </x:c>
       <x:c r="B6" s="4" t="str">
-        <x:v>Open Completed example. Every study, event, source excerpt, tool record, and action in that sheet is invented for teaching.</x:v>
+        <x:v>Read the Completed example. Published facts are cited to JOP. Proposed plans, practice errors, imagined comments, and AI-use records are labeled teaching exercises; they are not the authors’ original records.</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
         <x:v>Green = example</x:v>
@@ -453,12 +453,12 @@
         <x:v>Use approved storage</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="86" customHeight="1">
+    <x:row r="12" ht="150" customHeight="1">
       <x:c r="A12" s="11" t="str">
         <x:v>Sources / limits</x:v>
       </x:c>
       <x:c r="B12" s="4" t="str">
-        <x:v>Journal of Prosthodontics author instructions (checked 2026-09-08): https://onlinelibrary.wiley.com/page/journal/1532849x/homepage/forauthors.html</x:v>
+        <x:v>Xu B, Wang Y, Zhang L, Lin WS, Tan J, Chen L. Journal of Prosthodontics. 2026. Early View; supplied PDF pp. 1–7. Performance of a residual neural network system versus dental technicians for gingival porcelain shade matching https://onlinelibrary.wiley.com/doi/full/10.1111/jopr.70151 Methods, PDF pp. 2–4; Results and Tables 2–3, PDF pp. 4–6; Discussion, PDF p. 6.</x:v>
       </x:c>
       <x:c r="C12" s="4" t="str">
         <x:v>Recheck current guidance</x:v>
@@ -480,7 +480,7 @@
         <x:v>Calculation legend</x:v>
       </x:c>
       <x:c r="B14" s="4" t="str">
-        <x:v>Yellow cells are editable inputs; green cells on the example sheet contain invented entries. Dark teal total rows, if present, contain formulas. Do not replace formulas with typed totals.</x:v>
+        <x:v>Yellow cells are editable; green example cells contain published facts and clearly labeled teaching entries. Dark teal timing totals contain formulas. Preserve formulas when editing.</x:v>
       </x:c>
       <x:c r="C14" s="4" t="str">
         <x:v>No color-only status codes</x:v>
@@ -681,14 +681,14 @@
   <x:sheetData>
     <x:row r="1" ht="46" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>Example: language editing log</x:v>
+        <x:v>Example: teaching-use log for a shade-study paragraph</x:v>
       </x:c>
       <x:c r="B1" s="6"/>
       <x:c r="C1" s="6"/>
     </x:row>
     <x:row r="2" ht="47" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>COMPLETED EXAMPLE • Entirely hypothetical • Study this example, then complete your own blank sheet.</x:v>
+        <x:v>INVENTED ADMINISTRATIVE RECORD about teaching with Xu et al. This is not the authors’ AI-use disclosure.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -714,7 +714,7 @@
         <x:v>Record / project ID</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>TEACH-AI-001 / scanner manuscript teaching scenario</x:v>
+        <x:v>TEACH-XU-001. Fictional log of preparing a new educational paragraph about the published shade study.</x:v>
       </x:c>
       <x:c r="C5" s="4" t="str">
         <x:v>One record per tool use / task</x:v>
@@ -725,7 +725,7 @@
         <x:v>1. Tool name and provider</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Example Writing Assistant, Fictional Tools Ltd. — invented tool for this teaching record</x:v>
+        <x:v>ChatGPT, OpenAI (real service; this particular use record is invented for teaching).</x:v>
       </x:c>
       <x:c r="C6" s="4" t="str">
         <x:v>Record exact service and provider</x:v>
@@ -736,7 +736,7 @@
         <x:v>1. Model / version</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>1.0 (fictional version; not a real tool recommendation)</x:v>
+        <x:v>Model/version not displayed in this fictional scenario; unavailable recorded explicitly, not guessed.</x:v>
       </x:c>
       <x:c r="C7" s="4" t="str">
         <x:v>Record available version; never guess</x:v>
@@ -747,18 +747,18 @@
         <x:v>2. Date of use</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:v>46273</x:v>
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="C8" s="4" t="str">
         <x:v>Excel date; duplicate record for other dates</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="60" customHeight="1">
+    <x:row r="9" ht="69" customHeight="1">
       <x:c r="A9" s="11" t="str">
         <x:v>3. Application and extent</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Language editing and paragraph organization only; no new study claims, citations, or analyses requested.</x:v>
+        <x:v>Drafting and organization of one original educational Discussion paragraph using the verified Xu study summary; no new analysis or references.</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>Analysis, coding, editing, drafting, organization</x:v>
@@ -769,84 +769,84 @@
         <x:v>4. Specific sections / files</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>Introduction paragraphs 2–3 and Discussion paragraph 1, manuscript draft v3.</x:v>
+        <x:v>Journal-club handout: paragraph headed “Statistical improvement and clinical acceptability.” Not a section of the original Xu manuscript.</x:v>
       </x:c>
       <x:c r="C10" s="4" t="str">
         <x:v>Map tasks to manuscript locations</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="67" customHeight="1">
+    <x:row r="11" ht="69" customHeight="1">
       <x:c r="A11" s="11" t="str">
         <x:v>5. Accuracy validation completed</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>In this invented scenario, the lead author compared every edit with draft v3 and the verified claim-source map. A coauthor checked unchanged numbers, units, and citation IDs.</x:v>
+        <x:v>Invented completed check: the course presenter compared the paragraph with Xu Methods/Results and corrected an acceptability claim. A second reader checked 18/17 denominators and dimensionless ΔE00.</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>Who checked what, against which record?</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="101" customHeight="1">
+    <x:row r="12" ht="87" customHeight="1">
       <x:c r="A12" s="11" t="str">
         <x:v>6. Privacy / compliance safeguards</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>In this invented scenario, only team-owned nonconfidential teaching text was supplied. No human-subject, sensitive, or proprietary data were used. An institutional review had permitted this input class; access and retention settings were checked and documented. These actions are not claims about any real institution or tool.</x:v>
+        <x:v>Invented safeguards: only a permitted published-fact summary was entered; no individual measurements, scans, identifiers, proprietary material, or confidential review text. Service settings and institutional permission would need actual documentation in a real record.</x:v>
       </x:c>
       <x:c r="C12" s="4" t="str">
         <x:v>State actual authorization and controls</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="60" customHeight="1">
+    <x:row r="13" ht="69" customHeight="1">
       <x:c r="A13" s="11" t="str">
         <x:v>Permitted input description</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>Own teaching text only; no patient information, restricted sources, credentials, or confidential manufacturer specifications.</x:v>
+        <x:v>Aggregate published facts only: paired 18-volunteer design, three zones, overall values, thresholds, and the 17-volunteer subjective evaluation.</x:v>
       </x:c>
       <x:c r="C13" s="4" t="str">
         <x:v>Describe categories; do not paste restricted data</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="60" customHeight="1">
+    <x:row r="14" ht="69" customHeight="1">
       <x:c r="A14" s="11" t="str">
         <x:v>Prompt / output references</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>Approved project storage: prompts/TEACH-AI-001.txt; outputs/TEACH-AI-001.txt; edit-log-v1. These are illustrative file references.</x:v>
+        <x:v>Teaching prompt: website AI resources, ChatGPT example. Hypothetical retained files: TEACH-XU-001-prompt.txt and TEACH-XU-001-output.txt; they are illustrative references, not attached transcripts.</x:v>
       </x:c>
       <x:c r="C14" s="4" t="str">
         <x:v>Keep files in approved storage</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="60" customHeight="1">
+    <x:row r="15" ht="69" customHeight="1">
       <x:c r="A15" s="11" t="str">
         <x:v>Corrections and author decision</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>Rejected an unsupported “clinically superior” phrase; retained approved language edits and rechecked citation links.</x:v>
+        <x:v>In this fictional record, rejected “clinically acceptable matching” and retained the statement that both overall means exceeded 2.8. Kept the verified DOI with its claim.</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
         <x:v>Document changes actually accepted/rejected</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="60" customHeight="1">
+    <x:row r="16" ht="69" customHeight="1">
       <x:c r="A16" s="11" t="str">
         <x:v>Responsible reviewer</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>Lead author and reviewing coauthor (fictional roles); review documented 2026-09-08.</x:v>
+        <x:v>Course presenter and second reader (invented roles); fictional check date 9 September 2026. Replace with actual names and dates in a real project.</x:v>
       </x:c>
       <x:c r="C16" s="4" t="str">
         <x:v>Name the actual human reviewer</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="60" customHeight="1">
+    <x:row r="17" ht="69" customHeight="1">
       <x:c r="A17" s="11" t="str">
         <x:v>Disclosure location / status</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>Methods AI disclosure, linked to this log record. Check current journal instructions and any required additional detail before real submission.</x:v>
+        <x:v>For the teaching handout, disclose actual preparation use if applicable. For a real manuscript, reconcile all six fields with current journal instructions; do not use this log as the Xu authors’ disclosure.</x:v>
       </x:c>
       <x:c r="C17" s="4" t="str">
         <x:v>Reconcile with final manuscript</x:v>

</xml_diff>